<commit_message>
Fix generation Word: utiliser sys.executable pour python-docx sur Streamlit Cloud
</commit_message>
<xml_diff>
--- a/donnees_bons.xlsx
+++ b/donnees_bons.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L316"/>
+  <dimension ref="A1:L317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16936,6 +16936,68 @@
         </is>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>0304-BC-SHEA/NAP-2026</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>10:51:51</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>VLAVONOU PIERRE</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>+229 0197019848</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>KANDI</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>45MT</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>CF5600RB/CF5613RB</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>DAKOUDI SIMPLICE</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>17269/12</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>+229 0196147550</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Les modifications portés sur les fichiers
</commit_message>
<xml_diff>
--- a/donnees_bons.xlsx
+++ b/donnees_bons.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L317"/>
+  <dimension ref="A1:L316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16936,68 +16936,6 @@
         </is>
       </c>
     </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>0304-BC-SHEA/NAP-2026</t>
-        </is>
-      </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="C317" t="inlineStr">
-        <is>
-          <t>10:51:51</t>
-        </is>
-      </c>
-      <c r="D317" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="E317" t="inlineStr">
-        <is>
-          <t>VLAVONOU PIERRE</t>
-        </is>
-      </c>
-      <c r="F317" t="inlineStr">
-        <is>
-          <t>+229 0197019848</t>
-        </is>
-      </c>
-      <c r="G317" t="inlineStr">
-        <is>
-          <t>KANDI</t>
-        </is>
-      </c>
-      <c r="H317" t="inlineStr">
-        <is>
-          <t>45MT</t>
-        </is>
-      </c>
-      <c r="I317" t="inlineStr">
-        <is>
-          <t>CF5600RB/CF5613RB</t>
-        </is>
-      </c>
-      <c r="J317" t="inlineStr">
-        <is>
-          <t>DAKOUDI SIMPLICE</t>
-        </is>
-      </c>
-      <c r="K317" t="inlineStr">
-        <is>
-          <t>17269/12</t>
-        </is>
-      </c>
-      <c r="L317" t="inlineStr">
-        <is>
-          <t>+229 0196147550</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajout code QR haut droite sur bons de commande et paiement
</commit_message>
<xml_diff>
--- a/donnees_bons.xlsx
+++ b/donnees_bons.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L316"/>
+  <dimension ref="A1:L320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16936,6 +16936,254 @@
         </is>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>0304-BC-SHEA/NAP-2026</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>18:28:20</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>AHEGNI CASIMIR</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>+229 01 95249339</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>WASSA - PEHUNCO</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>50 MT</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>BR8467RB/BF4825RB</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>ALLASANE KASIME</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>01588 / 91 BOR</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>+229 01 43469015</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>0305-BC-SHEA/NAP-2026</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>18:30:48</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>AHEGNI CASIMIR</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>+229 0195249339</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>N'DALI &amp; TCHAOUROU</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>50 MT</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>BR5746RB/AT4393RB</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>DJEHA AIME</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>04448/2018 ZOU</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>+229 0196351801</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>0306-BC-SHEA/NAP-2026</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>18:32:58</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>AHEGNI CASMIR</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>+229 0195249339</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>BEMBEREKE</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>50T</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>BT8152RB</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>AKPO JOACHIM</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>97868511AC2</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>+229 01 42008350</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>0307-BC-SHEA/NAP-2026</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>18:37:12</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>AHEGNI CASIMIR</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>+229 0195249339</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>WASSA - PEHUNCO</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>50MT</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>BR8467RB/BF4825RB</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>ALLASANE KASIME</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>01588 / 91 BOR</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>+229 0143469015</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>